<commit_message>
fix: resolve guide overlap-vocabulary conflicts + 14533 T2 override + independent A/B review sheets
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/manifests/m3_pairs_draft.xlsx
+++ b/experiments/manifests/m3_pairs_draft.xlsx
@@ -8348,12 +8348,12 @@
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>검수: 'located'가 지리적 의미 — 같은 블록이면 T2로 adjudication</t>
+          <t>검수(2차): 두 질문 모두 'NASHVILLE, TENNESSEE' 같은 블록 참조 — T2 타당, adjudication 확정 요망</t>
         </is>
       </c>
       <c r="R94" t="b">

</xml_diff>